<commit_message>
Add Croatia predsjednik.hr scraper recipe
</commit_message>
<xml_diff>
--- a/data/sources/additional_master_sources.xlsx
+++ b/data/sources/additional_master_sources.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sources" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,6 +487,35 @@
       <c r="G2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>hrv_predsjednik</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Croatian</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Costa Rica presidencia recipe scaffold and source outbox row
</commit_message>
<xml_diff>
--- a/data/sources/additional_master_sources.xlsx
+++ b/data/sources/additional_master_sources.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sources" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,6 +487,35 @@
       <c r="G2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>cri_presidencia</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Spanish</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Armenia president recipe
</commit_message>
<xml_diff>
--- a/data/sources/additional_master_sources.xlsx
+++ b/data/sources/additional_master_sources.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,8 +516,6 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -550,7 +548,6 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>2015-12-10</t>
@@ -564,6 +561,40 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>NEW master row needed | country=Argentina; source_url=https://www.casarosada.gob.ar/informacion/discursos (Wayback/CDX); source_name=casarosada.gob.ar (Wayback); source_type=official_gov (archived); region=South America; iso3n=32; content_format=fulltext; leaders_covered=Kirchner-era (CFK, N. Kirchner). recipe recipes/arg_casarosada_wayback.yml on main (PR #9) — pagination: wayback over IA CDX, wayback_to 20151210 (complements live arg_casarosada from 2015-12-10 on); coverage ~2007–2015; FULL RUN underway.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>arm_president</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>recipe recipes/arm_president.yml — English press-release archive at /en/press-release/; web search confirmed h1/time/article structure and listing item URLs, but direct probe/run is blocked in this sandbox because president.am DNS does not resolve.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Cameroon PRC recipe
</commit_message>
<xml_diff>
--- a/data/sources/additional_master_sources.xlsx
+++ b/data/sources/additional_master_sources.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,8 +516,6 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -550,7 +548,6 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>2015-12-10</t>
@@ -564,6 +561,40 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>NEW master row needed | country=Argentina; source_url=https://www.casarosada.gob.ar/informacion/discursos (Wayback/CDX); source_name=casarosada.gob.ar (Wayback); source_type=official_gov (archived); region=South America; iso3n=32; content_format=fulltext; leaders_covered=Kirchner-era (CFK, N. Kirchner). recipe recipes/arg_casarosada_wayback.yml on main (PR #9) — pagination: wayback over IA CDX, wayback_to 20151210 (complements live arg_casarosada from 2015-12-10 on); coverage ~2007–2015; FULL RUN underway.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cmr_prc</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NEW master row needed | country=Cameroon; source_url=https://www.prc.cm/en/news/speeches-of-the-president; source_name=prc.cm; source_type=official_gov; region=Africa; iso3n=120; content_format=fulltext. recipe recipes/cmr_prc.yml on main — live probe/run blocked here by DNS resolution for prc.cm; candidate selectors from search results use .itemTitle/.itemDate/.itemFullText and start=10 pagination.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Belarus president.gov.by scraper recipe and status outbox row
</commit_message>
<xml_diff>
--- a/data/sources/additional_master_sources.xlsx
+++ b/data/sources/additional_master_sources.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sources" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,6 +494,7 @@
           <t>2026-06-29</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -564,6 +565,40 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>NEW master row needed | country=Argentina; source_url=https://www.casarosada.gob.ar/informacion/discursos (Wayback/CDX); source_name=casarosada.gob.ar (Wayback); source_type=official_gov (archived); region=South America; iso3n=32; content_format=fulltext; leaders_covered=Kirchner-era (CFK, N. Kirchner). recipe recipes/arg_casarosada_wayback.yml on main (PR #9) — pagination: wayback over IA CDX, wayback_to 20151210 (complements live arg_casarosada from 2015-12-10 on); coverage ~2007–2015; FULL RUN underway.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>blr_president</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Russian</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Recipe added at recipes/blr_president.yml. Validation blocked in this runner because president.gov.by DNS resolution fails ([Errno -5] No address associated with hostname), so probe/run returned 0 links.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Bhutan royalkidu recipe draft and source outbox row
</commit_message>
<xml_diff>
--- a/data/sources/additional_master_sources.xlsx
+++ b/data/sources/additional_master_sources.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sources" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,6 +494,7 @@
           <t>2026-06-29</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -564,6 +565,40 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>NEW master row needed | country=Argentina; source_url=https://www.casarosada.gob.ar/informacion/discursos (Wayback/CDX); source_name=casarosada.gob.ar (Wayback); source_type=official_gov (archived); region=South America; iso3n=32; content_format=fulltext; leaders_covered=Kirchner-era (CFK, N. Kirchner). recipe recipes/arg_casarosada_wayback.yml on main (PR #9) — pagination: wayback over IA CDX, wayback_to 20151210 (complements live arg_casarosada from 2015-12-10 on); coverage ~2007–2015; FULL RUN underway.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>btn_royalkidu</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NEW master row needed | country=Bhutan; source_url=https://www.royalkidu.bt/; source_name=royalkidu.bt; source_type=official_gov; region=Asia; content_format=fulltext. Recipe drafted in recipes/btn_royalkidu.yml, but runtime validation blocked in sandbox: DNS resolution failed for www.royalkidu.bt during probe and capped/full runs.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add draft Belgium monarchy recipe
</commit_message>
<xml_diff>
--- a/data/sources/additional_master_sources.xlsx
+++ b/data/sources/additional_master_sources.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,8 +516,6 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -550,7 +548,6 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>2015-12-10</t>
@@ -564,6 +561,38 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>NEW master row needed | country=Argentina; source_url=https://www.casarosada.gob.ar/informacion/discursos (Wayback/CDX); source_name=casarosada.gob.ar (Wayback); source_type=official_gov (archived); region=South America; iso3n=32; content_format=fulltext; leaders_covered=Kirchner-era (CFK, N. Kirchner). recipe recipes/arg_casarosada_wayback.yml on main (PR #9) — pagination: wayback over IA CDX, wayback_to 20151210 (complements live arg_casarosada from 2015-12-10 on); coverage ~2007–2015; FULL RUN underway.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>bel_monarchie</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NEW master row needed | country=Belgium; source_url=https://www.monarchie.be/en/monarchy/speeches; source_name=monarchie.be; source_type=official_gov; content_format=fulltext. recipe recipes/bel_monarchie.yml added, but live probe/run validation is blocked in this sandbox because monarchie.be DNS resolution fails; verify probe/capped/full run before marking validated.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Bangladesh Bangabhaban recipe draft
</commit_message>
<xml_diff>
--- a/data/sources/additional_master_sources.xlsx
+++ b/data/sources/additional_master_sources.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,8 +516,6 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -550,7 +548,6 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>2015-12-10</t>
@@ -564,6 +561,38 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>NEW master row needed | country=Argentina; source_url=https://www.casarosada.gob.ar/informacion/discursos (Wayback/CDX); source_name=casarosada.gob.ar (Wayback); source_type=official_gov (archived); region=South America; iso3n=32; content_format=fulltext; leaders_covered=Kirchner-era (CFK, N. Kirchner). recipe recipes/arg_casarosada_wayback.yml on main (PR #9) — pagination: wayback over IA CDX, wayback_to 20151210 (complements live arg_casarosada from 2015-12-10 on); coverage ~2007–2015; FULL RUN underway.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>bgd_bangabhaban</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Bengali</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NEW master row needed | country=Bangladesh; source_url=http://www.bangabhaban.gov.bd/; source_name=bangabhaban.gov.bd; source_type=official_gov; region=Asia; iso3n=50; content_format=fulltext. Added recipes/bgd_bangabhaban.yml as a Wayback-first recipe for the Bangladesh National Web Portal / Drupal speech archive (`/site/speech` plus legacy `/pages/pm-speeches` patterns). Sandbox DNS/network could not resolve bangabhaban.gov.bd or web.archive.org during authoring, so probe/full-run validation is still pending and the proposed status remains draft.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Belarus date attr and parsing for ISO datetimes
</commit_message>
<xml_diff>
--- a/data/sources/additional_master_sources.xlsx
+++ b/data/sources/additional_master_sources.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +48,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -494,7 +497,6 @@
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -517,8 +519,6 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -551,7 +551,6 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>2015-12-10</t>
@@ -589,16 +588,18 @@
           <t>Russian</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
+      <c r="E5" s="1" t="n">
+        <v>34945</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>46206</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Recipe added at recipes/blr_president.yml. Validation blocked in this runner because president.gov.by DNS resolution fails ([Errno -5] No address associated with hostname), so probe/run returned 0 links.</t>
+          <t>15-page --spread probe over sitemap discovery (~1,175 links) now parses dates after switching recipe date attr to data-datetime. Sampled pages span approximately 1995 through present.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
new sources and transcription note
</commit_message>
<xml_diff>
--- a/data/sources/additional_master_sources.xlsx
+++ b/data/sources/additional_master_sources.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sources" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,6 +494,7 @@
           <t>2026-06-29</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -564,6 +565,142 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>NEW master row needed | country=Argentina; source_url=https://www.casarosada.gob.ar/informacion/discursos (Wayback/CDX); source_name=casarosada.gob.ar (Wayback); source_type=official_gov (archived); region=South America; iso3n=32; content_format=fulltext; leaders_covered=Kirchner-era (CFK, N. Kirchner). recipe recipes/arg_casarosada_wayback.yml on main (PR #9) — pagination: wayback over IA CDX, wayback_to 20151210 (complements live arg_casarosada from 2015-12-10 on); coverage ~2007–2015; FULL RUN underway.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ind_pmindia</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>English/Hindi</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NEW master row needed | country=India; source_url=https://www.pmindia.gov.in/en/; source_name=pmindia.gov.in; source_type=official_gov; region=Asia; iso3n=356; content_format=fulltext. PM Modi is India's actual national leader (the President in master is ceremonial). The /en/speeches/ section is largely video; look for text under /en/pms-speeches/ or fall back to narendramodi.in/category/text-speeches. GitHub issue #43 already opened - do NOT re-run create_issues_from_master.py for this row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>tha_thaigov</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Thai/English</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>NEW master row needed | country=Thailand; source_url=https://www.thaigov.go.th/en/news; source_name=thaigov.go.th; source_type=official_gov; region=Asia; iso3n=764; content_format=fulltext. Royal Thai Government news portal carrying PM statements/speeches (the Royal Office in master is the ceremonial monarchy). English + Thai listings. GitHub issue #44 already opened - do NOT re-run create_issues_from_master.py for this row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>idn_setkab</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>English (+Indonesian)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>NEW master row needed | country=Indonesia; source_url=https://setkab.go.id/en/category/speech-transcript/; source_name=setkab.go.id; source_type=official_gov; region=Asia; iso3n=360; content_format=fulltext. Cabinet Secretariat 'Speech Transcript' archive: ~200 pages of full presidential transcripts, WordPress-style /page/N/ pagination. SSL cert chain does not verify -&gt; likely needs verify_ssl: false. Indonesian-language originals at setkab.go.id/kategori/. GitHub issue #45 already opened - do NOT re-run create_issues_from_master.py for this row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>phl_pco</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>static/js</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>English/Filipino</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>NEW master row needed | country=Philippines; source_url=https://pco.gov.ph/presidential-speech/; source_name=pco.gov.ph; source_type=official_gov; region=Asia; iso3n=608; content_format=fulltext. Presidential Communications Office 'Presidential Speeches' (Marcos Jr.), /page/N/ pagination. Returns HTTP 403 to the bot UA (WAF) -&gt; likely needs a browser user_agent override (cf. recipes/col_presidencia.yml). Scraper-friendlier historical alternative: https://www.officialgazette.gov.ph/section/historical-papers-documents/speeches/. GitHub issue #46 already opened - do NOT re-run create_issues_from_master.py for this row.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update ind_pmindia outbox row
</commit_message>
<xml_diff>
--- a/data/sources/additional_master_sources.xlsx
+++ b/data/sources/additional_master_sources.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +48,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -494,7 +497,6 @@
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -517,8 +519,6 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -551,7 +551,6 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>2015-12-10</t>
@@ -576,7 +575,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -589,16 +588,12 @@
           <t>English/Hindi</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
+      <c r="G5" s="1" t="n">
+        <v>46206</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NEW master row needed | country=India; source_url=https://www.pmindia.gov.in/en/; source_name=pmindia.gov.in; source_type=official_gov; region=Asia; iso3n=356; content_format=fulltext. PM Modi is India's actual national leader (the President in master is ceremonial). The /en/speeches/ section is largely video; look for text under /en/pms-speeches/ or fall back to narendramodi.in/category/text-speeches. GitHub issue #43 already opened - do NOT re-run create_issues_from_master.py for this row.</t>
+          <t>NEW master row needed | country=India; source_url=https://www.pmindia.gov.in/en/; source_name=pmindia.gov.in; source_type=official_gov; region=Asia; iso3n=356; content_format=fulltext. PM Modi is India's actual national leader (the President in master is ceremonial). Recipe recipes/ind_pmindia.yml targets the PMIndia WordPress speech archives (/en/tag/pmspeech and /en/category/pms-speeches). Live validation is still pending because pmindia.gov.in did not resolve in this runner during probe.</t>
         </is>
       </c>
     </row>
@@ -623,8 +618,6 @@
           <t>Thai/English</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>2026-07-03</t>
@@ -657,8 +650,6 @@
           <t>English (+Indonesian)</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>2026-07-03</t>
@@ -691,8 +682,6 @@
           <t>English/Filipino</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>2026-07-03</t>

</xml_diff>

<commit_message>
Add idn_setkab recipe and outbox status update
</commit_message>
<xml_diff>
--- a/data/sources/additional_master_sources.xlsx
+++ b/data/sources/additional_master_sources.xlsx
@@ -644,7 +644,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>none</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>NEW master row needed | country=Indonesia; source_url=https://setkab.go.id/en/category/speech-transcript/; source_name=setkab.go.id; source_type=official_gov; region=Asia; iso3n=360; content_format=fulltext. Cabinet Secretariat 'Speech Transcript' archive: ~200 pages of full presidential transcripts, WordPress-style /page/N/ pagination. SSL cert chain does not verify -&gt; likely needs verify_ssl: false. Indonesian-language originals at setkab.go.id/kategori/. GitHub issue #45 already opened - do NOT re-run create_issues_from_master.py for this row.</t>
+          <t>NEW master row needed | country=Indonesia; source_url=https://setkab.go.id/en/category/speech-transcript/; source_name=setkab.go.id; source_type=official_gov; region=Asia; iso3n=360; content_format=fulltext. Cabinet Secretariat 'Speech Transcript' archive: ~200 pages of full presidential transcripts, WordPress-style /page/N/ pagination. SSL cert chain does not verify -&gt; likely needs verify_ssl: false. Indonesian-language originals at setkab.go.id/kategori/. GitHub issue #45 already opened - do NOT re-run create_issues_from_master.py for this row. Recipe file recipes/idn_setkab.yml added. Probe and capped/full runs in this sandbox could not reach setkab.go.id (DNS resolution failure: [Errno -5] No address associated with hostname), so validation remains pending.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Philippines PCO scraper recipe
</commit_message>
<xml_diff>
--- a/data/sources/additional_master_sources.xlsx
+++ b/data/sources/additional_master_sources.xlsx
@@ -494,7 +494,6 @@
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -517,8 +516,6 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -551,7 +548,6 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>2015-12-10</t>
@@ -589,8 +585,6 @@
           <t>English/Hindi</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>2026-07-03</t>
@@ -623,8 +617,6 @@
           <t>Thai/English</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>2026-07-03</t>
@@ -657,8 +649,6 @@
           <t>English (+Indonesian)</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>2026-07-03</t>
@@ -678,12 +668,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>static/js</t>
+          <t>js</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -691,8 +681,6 @@
           <t>English/Filipino</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>2026-07-03</t>
@@ -700,7 +688,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>NEW master row needed | country=Philippines; source_url=https://pco.gov.ph/presidential-speech/; source_name=pco.gov.ph; source_type=official_gov; region=Asia; iso3n=608; content_format=fulltext. Presidential Communications Office 'Presidential Speeches' (Marcos Jr.), /page/N/ pagination. Returns HTTP 403 to the bot UA (WAF) -&gt; likely needs a browser user_agent override (cf. recipes/col_presidencia.yml). Scraper-friendlier historical alternative: https://www.officialgazette.gov.ph/section/historical-papers-documents/speeches/. GitHub issue #46 already opened - do NOT re-run create_issues_from_master.py for this row.</t>
+          <t>NEW master row needed | country=Philippines; source_url=https://pco.gov.ph/presidential-speech/; source_name=pco.gov.ph; source_type=official_gov; region=Asia; iso3n=608; content_format=fulltext. recipe recipes/phl_pco.yml added for issue #46 using renderer:js + browser user_agent + /page/N/ pagination; selectors based on external scraper evidence (.clamp-4, .release-date, .release-content p). Local validation: recipe loads and tests pass. Live probe and capped/full crawl attempts from this sandbox failed at DNS resolution with ERR_NAME_NOT_RESOLVED for pco.gov.ph, so the row remains draft pending validation from a network that can resolve the host.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply reviewer fixes to blr_president recipe; drop advisory outbox row
Probe-verified corrections (see PR #36 review):
- Broaden link_pattern to /ru/events/<slug> (drop the \d{10} requirement): only
  ~8% of events carry a trailing id, so the old pattern silently dropped ~92% of
  speeches incl. all pre-2021 history.
- Crawl sitemap.event.xml directly instead of the index (which pulls 8 unrelated
  child sitemaps); fix the 404 /ru/events/addresses start_url.
- --spread probe: 14,471 links, title/text/date OK across 2007-2026.

Revert the outbox xlsx to origin/main (drops #36's advisory blr_president row) so the
binary file no longer conflicts; the source is validated in master_sources.xlsx at merge.
(Outbox is migrating to a union-merged CSV on main; see the review_workflow/(b) change.)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/sources/additional_master_sources.xlsx
+++ b/data/sources/additional_master_sources.xlsx
@@ -16,9 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -48,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,6 +494,7 @@
           <t>2026-06-29</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -519,6 +517,8 @@
           <t>Spanish</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -551,6 +551,7 @@
           <t>Spanish</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>2015-12-10</t>
@@ -570,12 +571,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>blr_president</t>
+          <t>ind_pmindia</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -585,21 +586,121 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Russian</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>34945</v>
-      </c>
-      <c r="F5" s="1" t="n">
-        <v>46206</v>
-      </c>
-      <c r="G5" s="1" t="n">
-        <v>46206</v>
+          <t>English/Hindi</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>15-page --spread probe over sitemap discovery (~1,175 links) now parses dates after switching recipe date attr to data-datetime. Sampled pages span approximately 1995 through present.</t>
+          <t>NEW master row needed | country=India; source_url=https://www.pmindia.gov.in/en/; source_name=pmindia.gov.in; source_type=official_gov; region=Asia; iso3n=356; content_format=fulltext. PM Modi is India's actual national leader (the President in master is ceremonial). The /en/speeches/ section is largely video; look for text under /en/pms-speeches/ or fall back to narendramodi.in/category/text-speeches. GitHub issue #43 already opened - do NOT re-run create_issues_from_master.py for this row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>tha_thaigov</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Thai/English</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>NEW master row needed | country=Thailand; source_url=https://www.thaigov.go.th/en/news; source_name=thaigov.go.th; source_type=official_gov; region=Asia; iso3n=764; content_format=fulltext. Royal Thai Government news portal carrying PM statements/speeches (the Royal Office in master is the ceremonial monarchy). English + Thai listings. GitHub issue #44 already opened - do NOT re-run create_issues_from_master.py for this row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>idn_setkab</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>English (+Indonesian)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>NEW master row needed | country=Indonesia; source_url=https://setkab.go.id/en/category/speech-transcript/; source_name=setkab.go.id; source_type=official_gov; region=Asia; iso3n=360; content_format=fulltext. Cabinet Secretariat 'Speech Transcript' archive: ~200 pages of full presidential transcripts, WordPress-style /page/N/ pagination. SSL cert chain does not verify -&gt; likely needs verify_ssl: false. Indonesian-language originals at setkab.go.id/kategori/. GitHub issue #45 already opened - do NOT re-run create_issues_from_master.py for this row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>phl_pco</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>static/js</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>English/Filipino</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>NEW master row needed | country=Philippines; source_url=https://pco.gov.ph/presidential-speech/; source_name=pco.gov.ph; source_type=official_gov; region=Asia; iso3n=608; content_format=fulltext. Presidential Communications Office 'Presidential Speeches' (Marcos Jr.), /page/N/ pagination. Returns HTTP 403 to the bot UA (WAF) -&gt; likely needs a browser user_agent override (cf. recipes/col_presidencia.yml). Scraper-friendlier historical alternative: https://www.officialgazette.gov.ph/section/historical-papers-documents/speeches/. GitHub issue #46 already opened - do NOT re-run create_issues_from_master.py for this row.</t>
         </is>
       </c>
     </row>

</xml_diff>